<commit_message>
Update to most recent DS
</commit_message>
<xml_diff>
--- a/mortality/data_processing_elements_mortality-BCS.xlsx
+++ b/mortality/data_processing_elements_mortality-BCS.xlsx
@@ -1,29 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Other computers\My Computer\twey working files\ProPASS\BCS\DPEs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\twey\OneDrive\Bureau\twey working files\ProPASS\BCS\DPEs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CB8A655-9093-4BD8-B568-A1D8C046F204}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7498068C-C77A-418F-91A3-AF1E3EFB3BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AB$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AB$12</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="96">
   <si>
     <t>index</t>
   </si>
@@ -296,6 +309,30 @@
   </si>
   <si>
     <t>outcme11</t>
+  </si>
+  <si>
+    <t>adm_months_followup</t>
+  </si>
+  <si>
+    <t>Months of follow-up</t>
+  </si>
+  <si>
+    <t>Number of months of participant follow-up from baseline</t>
+  </si>
+  <si>
+    <t>months</t>
+  </si>
+  <si>
+    <t>participant</t>
+  </si>
+  <si>
+    <t>at data collection</t>
+  </si>
+  <si>
+    <t>cohort documentation</t>
+  </si>
+  <si>
+    <t>If this is calculated from difference between two dates, round to nearest whole month.</t>
   </si>
 </sst>
 </file>
@@ -736,40 +773,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BM11"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:BM12"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.7265625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="15.7265625" style="8" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.54296875" style="8" customWidth="1"/>
-    <col min="4" max="4" width="31.1796875" style="8" customWidth="1"/>
-    <col min="5" max="5" width="32.26953125" style="8" customWidth="1"/>
-    <col min="6" max="6" width="7.1796875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="3.7109375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="15.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" style="8" customWidth="1"/>
+    <col min="5" max="5" width="32.28515625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="7.140625" style="8" customWidth="1"/>
     <col min="7" max="9" width="6" style="8" customWidth="1"/>
-    <col min="10" max="10" width="28.81640625" style="8" customWidth="1"/>
-    <col min="11" max="11" width="21.54296875" style="8" customWidth="1"/>
-    <col min="12" max="12" width="22.81640625" style="9" customWidth="1"/>
-    <col min="13" max="13" width="17.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="28.85546875" style="8" customWidth="1"/>
+    <col min="11" max="11" width="21.5703125" style="8" customWidth="1"/>
+    <col min="12" max="12" width="22.85546875" style="9" customWidth="1"/>
+    <col min="13" max="13" width="17.140625" style="8" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="27" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28.54296875" style="10" customWidth="1"/>
-    <col min="16" max="16" width="7.1796875" style="8" customWidth="1"/>
-    <col min="17" max="17" width="24.453125" style="8" customWidth="1"/>
-    <col min="18" max="18" width="11.81640625" style="8" customWidth="1"/>
-    <col min="19" max="19" width="12.1796875" style="8" customWidth="1"/>
+    <col min="15" max="15" width="28.5703125" style="10" customWidth="1"/>
+    <col min="16" max="16" width="7.140625" style="8" customWidth="1"/>
+    <col min="17" max="17" width="24.42578125" style="8" customWidth="1"/>
+    <col min="18" max="18" width="11.85546875" style="8" customWidth="1"/>
+    <col min="19" max="19" width="12.140625" style="8" customWidth="1"/>
     <col min="20" max="20" width="15" style="8" customWidth="1"/>
-    <col min="21" max="21" width="34.7265625" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="34.7109375" style="8" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="20" style="10" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="31.54296875" style="10" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="21.81640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="31.7265625" style="8" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="27.453125" style="8" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="16.1796875" style="8" customWidth="1"/>
-    <col min="28" max="28" width="14.26953125" style="8" customWidth="1"/>
+    <col min="23" max="23" width="31.5703125" style="10" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="21.85546875" style="10" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="31.7109375" style="8" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="27.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="16.140625" style="8" customWidth="1"/>
+    <col min="28" max="28" width="14.28515625" style="8" customWidth="1"/>
     <col min="29" max="29" width="9" style="8" customWidth="1"/>
     <col min="30" max="16384" width="9" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -855,7 +892,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="2" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A2" s="8">
         <v>1</v>
       </c>
@@ -898,7 +935,7 @@
       </c>
       <c r="X2" s="8"/>
     </row>
-    <row r="3" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>2</v>
       </c>
@@ -938,7 +975,7 @@
       </c>
       <c r="X3" s="8"/>
     </row>
-    <row r="4" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>3</v>
       </c>
@@ -978,7 +1015,7 @@
       </c>
       <c r="X4" s="8"/>
     </row>
-    <row r="5" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>4</v>
       </c>
@@ -1015,7 +1052,7 @@
       </c>
       <c r="X5" s="8"/>
     </row>
-    <row r="6" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <v>5</v>
       </c>
@@ -1065,7 +1102,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="7" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>6</v>
       </c>
@@ -1113,7 +1150,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="8" spans="1:65" ht="130.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>7</v>
       </c>
@@ -1121,92 +1158,53 @@
         <v>77</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>54</v>
+        <v>88</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>55</v>
+        <v>89</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>56</v>
+        <v>90</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>47</v>
       </c>
+      <c r="G8" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>92</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>94</v>
+      </c>
       <c r="L8" s="9" t="s">
-        <v>51</v>
+        <v>95</v>
       </c>
       <c r="M8" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="N8" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="O8" s="7" t="s">
-        <v>78</v>
-      </c>
-      <c r="P8" s="8" t="s">
-        <v>58</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="N8" s="9"/>
+      <c r="O8" s="8"/>
+      <c r="Q8" s="9"/>
       <c r="R8" s="8" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="S8" s="8" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="T8" s="8" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="U8" s="8" t="s">
-        <v>79</v>
-      </c>
-      <c r="W8" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="Y8" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="Z8" s="10"/>
-      <c r="AA8" s="10"/>
-      <c r="AB8" s="10"/>
-      <c r="AC8" s="10"/>
-      <c r="AD8" s="10"/>
-      <c r="AE8" s="10"/>
-      <c r="AF8" s="10"/>
-      <c r="AG8" s="10"/>
-      <c r="AH8" s="10"/>
-      <c r="AI8" s="10"/>
-      <c r="AJ8" s="10"/>
-      <c r="AK8" s="10"/>
-      <c r="AL8" s="10"/>
-      <c r="AM8" s="10"/>
-      <c r="AN8" s="10"/>
-      <c r="AO8" s="10"/>
-      <c r="AP8" s="10"/>
-      <c r="AQ8" s="10"/>
-      <c r="AR8" s="10"/>
-      <c r="AS8" s="10"/>
-      <c r="AT8" s="10"/>
-      <c r="AU8" s="10"/>
-      <c r="AV8" s="10"/>
-      <c r="AW8" s="10"/>
-      <c r="AX8" s="10"/>
-      <c r="AY8" s="10"/>
-      <c r="AZ8" s="10"/>
-      <c r="BA8" s="10"/>
-      <c r="BB8" s="10"/>
-      <c r="BC8" s="10"/>
-      <c r="BD8" s="10"/>
-      <c r="BE8" s="10"/>
-      <c r="BF8" s="10"/>
-      <c r="BG8" s="10"/>
-      <c r="BH8" s="10"/>
-      <c r="BI8" s="10"/>
-      <c r="BJ8" s="10"/>
-      <c r="BK8" s="10"/>
-      <c r="BL8" s="10"/>
-      <c r="BM8" s="10"/>
+        <v>52</v>
+      </c>
+      <c r="X8" s="8"/>
     </row>
-    <row r="9" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:65" ht="135" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>8</v>
       </c>
@@ -1214,33 +1212,50 @@
         <v>77</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="F9" s="8" t="s">
         <v>47</v>
       </c>
+      <c r="L9" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="M9" s="8" t="s">
-        <v>40</v>
+        <v>87</v>
+      </c>
+      <c r="N9" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="P9" s="8" t="s">
+        <v>58</v>
       </c>
       <c r="R9" s="8" t="s">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="S9" s="8" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="T9" s="8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="U9" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="Y9" s="10"/>
+        <v>79</v>
+      </c>
+      <c r="W9" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Y9" s="10" t="s">
+        <v>81</v>
+      </c>
       <c r="Z9" s="10"/>
       <c r="AA9" s="10"/>
       <c r="AB9" s="10"/>
@@ -1282,7 +1297,7 @@
       <c r="BL9" s="10"/>
       <c r="BM9" s="10"/>
     </row>
-    <row r="10" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>9</v>
       </c>
@@ -1290,13 +1305,13 @@
         <v>77</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10" s="8" t="s">
         <v>47</v>
@@ -1304,7 +1319,6 @@
       <c r="M10" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="O10" s="8"/>
       <c r="R10" s="8" t="s">
         <v>52</v>
       </c>
@@ -1359,7 +1373,7 @@
       <c r="BL10" s="10"/>
       <c r="BM10" s="10"/>
     </row>
-    <row r="11" spans="1:65" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:65" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>10</v>
       </c>
@@ -1367,13 +1381,13 @@
         <v>77</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F11" s="8" t="s">
         <v>47</v>
@@ -1436,10 +1450,87 @@
       <c r="BL11" s="10"/>
       <c r="BM11" s="10"/>
     </row>
+    <row r="12" spans="1:65" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="O12" s="8"/>
+      <c r="R12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="S12" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="T12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="U12" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="Y12" s="10"/>
+      <c r="Z12" s="10"/>
+      <c r="AA12" s="10"/>
+      <c r="AB12" s="10"/>
+      <c r="AC12" s="10"/>
+      <c r="AD12" s="10"/>
+      <c r="AE12" s="10"/>
+      <c r="AF12" s="10"/>
+      <c r="AG12" s="10"/>
+      <c r="AH12" s="10"/>
+      <c r="AI12" s="10"/>
+      <c r="AJ12" s="10"/>
+      <c r="AK12" s="10"/>
+      <c r="AL12" s="10"/>
+      <c r="AM12" s="10"/>
+      <c r="AN12" s="10"/>
+      <c r="AO12" s="10"/>
+      <c r="AP12" s="10"/>
+      <c r="AQ12" s="10"/>
+      <c r="AR12" s="10"/>
+      <c r="AS12" s="10"/>
+      <c r="AT12" s="10"/>
+      <c r="AU12" s="10"/>
+      <c r="AV12" s="10"/>
+      <c r="AW12" s="10"/>
+      <c r="AX12" s="10"/>
+      <c r="AY12" s="10"/>
+      <c r="AZ12" s="10"/>
+      <c r="BA12" s="10"/>
+      <c r="BB12" s="10"/>
+      <c r="BC12" s="10"/>
+      <c r="BD12" s="10"/>
+      <c r="BE12" s="10"/>
+      <c r="BF12" s="10"/>
+      <c r="BG12" s="10"/>
+      <c r="BH12" s="10"/>
+      <c r="BI12" s="10"/>
+      <c r="BJ12" s="10"/>
+      <c r="BK12" s="10"/>
+      <c r="BL12" s="10"/>
+      <c r="BM12" s="10"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AB11" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AB11">
-      <sortCondition ref="A1:A11"/>
+  <autoFilter ref="A1:AB12" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AB12">
+      <sortCondition ref="A1:A12"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>